<commit_message>
fix: add inference report topic body content
</commit_message>
<xml_diff>
--- a/inference-report/推理token工厂汇报大纲_汇报版_v2.0.xlsx
+++ b/inference-report/推理token工厂汇报大纲_汇报版_v2.0.xlsx
@@ -1274,7 +1274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1403,8 +1403,191 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="6" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>MOE 专家并行验证计划</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>正文口径</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>状态/资源</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>验证结论</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>MOE 专家并行需要验证测试，用于确认 GLM 大参数 MOE 在多卡专家切分下的吞吐和延迟边界。</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>需要验证测试。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>资源申请</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>资源申请按 GLM5.1 或 GLM5.2 FP8 部署口径，优先申请可支撑多 GPU Experts 的 H200 资源。</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>GLM5.1 或 GLM5.2 FP8 资源待申请。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>EP 原理</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Router 将 token 分配给不同专家，专家切分到多 GPU Experts 上执行，再通过 All2All 完成跨卡交换和聚合。</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>重点关注跨卡通信是否成为瓶颈。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>指标与资源申请</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>验证内容</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>专家切分</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>对比不同专家切分和专家副本策略。</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>吞吐、TTFT、TPOT。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>多 GPU Experts</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>验证专家分布在多卡后的负载均衡和显存压力。</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>显存水位、GPU 利用率。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>All2All</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>记录跨卡 All2All 通信量、等待时间和抖动。</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>跨卡通信、TPOT。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>端到端收益</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>和非 EP 或单机基线对比，判断是否支撑 GLM5.1/GLM5.2 FP8 部署。</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>吞吐、TTFT、TPOT、显存水位。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -1418,7 +1601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1547,8 +1730,108 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="6" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Continuous Batching 能力说明</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>正文口径</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>状态/影响</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>能力状态</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>连续批处理为框架原生支持能力，当前调度默认依赖该能力。</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>已具备。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>测试范围</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>该能力无法关闭，且无需独立测试；本期不作为独立测试项。</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>无法关闭/无需独立测试。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>汇报口径</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>只作为已具备能力说明，不单独申请资源或产出专项收益结论。</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>作为基线能力写入汇总。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>对基线影响</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Continuous Batching 会作为并发吞吐基线前提，影响请求合批、排队和 decode 调度表现。</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>解读并发吞吐时需说明该前提。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -1562,7 +1845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1630,8 +1913,155 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>面向领导的优先级建议</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>建议项</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>领导汇报口径</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>下一步</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>FP8/量化优先落地</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>H200 历史数据已支撑 FP8/量化作为近期最确定的容量收益方向。</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>优先推进 GLM5.1/GLM5.2 FP8 部署口径和峰值场景复测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Prefix/KV 命中补系统数据</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>机制结论明确，但需要系统数据补齐 prefix_ratio、cache hit rate、TTFT 降幅和吞吐。</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>安排胡正升完成不同上下文/并发组合补测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>PD 分离申请异构资源验证</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>PD 分离需要 H200 做 P、H20 做 D 的异构资源验证，确认长上下文 Prefill 与 Decode 拆分收益。</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>申请 H200+H20 资源并按三组基线跑端到端压测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>MOE EP 按 GLM5.1/GLM5.2 FP8 申请资源验证</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>MOE 专家并行需要按 GLM5.1/GLM5.2 FP8 部署资源验证专家切分、All2All 和跨卡通信成本。</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>申请多 GPU Experts 资源并补充吞吐、TTFT、TPOT、显存水位。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Continuous Batching 已具备</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>连续批处理为框架原生支持，无法关闭且无需独立测试。</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>作为并发吞吐基线前提写入能力说明。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A7:H7"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2929,7 +3359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3058,8 +3488,208 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="6" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>KV Cache 量化结论与补测方向</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>正文口径</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>状态/下一步</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>H200 已有口径</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>H200 上 fp8 vs fp16/bf16 类 KV Cache 量化已有结论口径：KV 显存节省约 50%。</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>有结论但缺系统数据/后续补测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>收益数据缺口</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>吞吐/延迟收益待胡正升补齐系统测试数据，或以现有历史数据补录同口径对比。</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>补齐后再写 TPS/Tokens/s、TTFT、TPOT/平均延迟收益。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>fp4 范围</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>fp4 因 H200 不支持，本期暂不测；汇报中只说明硬件限制，不作为本期收益结论。</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>本期不纳入测试矩阵。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>验证指标</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>验证目的</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>当前口径</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>TPS/Tokens/s</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>验证吞吐是否随 KV Cache 量化提升。</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>待胡正升补齐系统测试数据。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>TTFT</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>验证 prefill 和 KV 分配对首 token 延迟的影响。</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>待补测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>TPOT/平均延迟</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>验证 decode 阶段平均生成延迟是否下降。</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>待补测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>显存水位</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>确认 KV 显存节省约 50% 是否反映到实际 GPU 显存水位。</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>已有结论但缺系统数据。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>gpu_cache_utilization</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>观察 cache 使用率和水位变化，避免只看理论节省。</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>后续补测。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -3073,7 +3703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3202,8 +3832,108 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="6" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Prefix/KV 命中结论与后续补测</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>正文口径</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>状态/验证方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>当前状态</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Prefix/KV 命中已有机制结论，但缺少端到端系统压测数据。</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>有结论但缺系统数据，必须安排后续补测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>验证变量</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>按 prefix_ratio 分层构造共享前缀请求，统计 cache hit rate 和 GPU cache 命中变化。</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>覆盖不同上下文长度和不同并发组合。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>收益指标</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>重点验证 TTFT 降幅、吞吐提升和 GPU cache 命中变化，避免只用单一命中率说明收益。</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>后续补测需同时记录 prefix_ratio、cache hit rate、TTFT、吞吐。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>组合矩阵</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>短/中/长上下文分别叠加低/中/高并发，观察前缀复用在并发压力下是否稳定。</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>输出不同上下文/并发组合的对比表。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -3217,7 +3947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3346,8 +4076,108 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="6" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>投机解码原理与测试方案</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>主题</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>正文口径</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>状态/指标</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>原理</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>draft 模型先生成候选 token，目标模型批量 Verify 后接受或拒绝候选，收益来自减少目标模型逐 token 调用次数。</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>待胡正升测试返回。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>候选配置</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>测试候选 token 1/3/5，分别观察低候选和高候选下的吞吐、延迟和回退成本。</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>候选 token 1/3/5 为本轮固定对比项。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>核心指标</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>关注接受率、TPS/Tokens/s、TTFT、TPOT/平均延迟，并记录高并发衰减。</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>接受率偏低时需同步解释 TPOT 收益下降原因。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>并发压力</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>低/中/高并发分别测试，观察 draft 模型开销、Verify 批处理和调度开销是否抵消收益。</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>待胡正升测试返回。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>